<commit_message>
PLP Urls and FF quit logic update
</commit_message>
<xml_diff>
--- a/src/main/resources/AllCollectionPages.xlsx
+++ b/src/main/resources/AllCollectionPages.xlsx
@@ -1,19 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23901"/>
+  <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vijeta\git\TJ_Automation\src\main\resources\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D47F69B-B8AA-48C7-B973-A8C18FCD3F65}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15210" windowHeight="4995"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$A$62</definedName>
   </definedNames>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -23,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="98">
   <si>
     <t>https://tommyjohn.com/collections/mens-new-arrivals-1</t>
   </si>
@@ -46,12 +51,6 @@
     <t>https://tommyjohn.com/collections/all-clothing</t>
   </si>
   <si>
-    <t>https://tommyjohn.com/collections/mens-tees-polos</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/pants-and-shorts</t>
-  </si>
-  <si>
     <t>https://tommyjohn.com/collections/clothing-packs</t>
   </si>
   <si>
@@ -121,18 +120,9 @@
     <t>https://tommyjohn.com/collections/youth-socks-men-section</t>
   </si>
   <si>
-    <t>https://tommyjohn.com/collections/sweaters-sweatshirts-1</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/jackets-outerwear-1</t>
-  </si>
-  <si>
     <t>https://tommyjohn.com/collections/all-womens</t>
   </si>
   <si>
-    <t>https://tommyjohn.com/collections/sale</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://tommyjohn.com/collections/mens-underwear </t>
   </si>
   <si>
@@ -142,9 +132,6 @@
     <t xml:space="preserve">https://tommyjohn.com/collections/loungewear </t>
   </si>
   <si>
-    <t>https://tommyjohn.com/collections/mens-sale</t>
-  </si>
-  <si>
     <t>https://tommyjohn.com/collections/new-arrivals-mens-underwear</t>
   </si>
   <si>
@@ -199,30 +186,6 @@
     <t>https://tommyjohn.com/collections/mens-lounge-sleep-tops</t>
   </si>
   <si>
-    <t>https://tommyjohn.com/collections/mens-sale-tees-polos</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/mens-sale-undershirts</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/mens-sale-sweaters-jackets</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/mens-sale-button-downs</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/mens-sale-socks</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/mens-sale-underwear</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/mens-sale-lounge-sleep</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/mens-sale-clothing</t>
-  </si>
-  <si>
     <t>https://tommyjohn.com/collections/mens-shirts</t>
   </si>
   <si>
@@ -328,15 +291,6 @@
     <t>https://tommyjohn.com/collections/gift-cards</t>
   </si>
   <si>
-    <t>https://tommyjohn.com/collections/gift-guide-men</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/gift-guide-women</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/gift-guide-dual-gender</t>
-  </si>
-  <si>
     <t>https://tommyjohn.com/collections/new-arrivals-mens</t>
   </si>
   <si>
@@ -361,43 +315,19 @@
     <t>https://tommyjohn.com/collections/loungewear-womens</t>
   </si>
   <si>
-    <t>https://tommyjohn.com/collections/womens-lounge-bottoms</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/womens-lounge-tops</t>
-  </si>
-  <si>
     <t>https://tommyjohn.com/collections/pajamas-womens</t>
   </si>
   <si>
     <t>https://tommyjohn.com/collections/bralette-packs</t>
   </si>
   <si>
-    <t>https://tommyjohn.com/collections/womens-work-from-home</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/womens-work-from-home-loungewear</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/womens-work-from-home-underwear</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/womens-work-from-home-clothing</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/gifts-under-25-all</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/gifts-under-50-all</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/gifts-under-75-all</t>
+    <t>URLs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -756,636 +686,512 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A123"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:A98"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="98.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="98.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
-        <v>122</v>
-      </c>
-    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A9" r:id="rId1"/>
-    <hyperlink ref="A10" r:id="rId2"/>
-    <hyperlink ref="A11" r:id="rId3"/>
-    <hyperlink ref="A13" r:id="rId4"/>
-    <hyperlink ref="A1" r:id="rId5"/>
-    <hyperlink ref="A17" r:id="rId6"/>
+    <hyperlink ref="A6" r:id="rId1" xr:uid="{98E17712-DE89-4F4D-8F98-F76F0031EF2F}"/>
+    <hyperlink ref="A7" r:id="rId2" xr:uid="{D2385662-B314-419A-B5D8-DF106799304E}"/>
+    <hyperlink ref="A8" r:id="rId3" xr:uid="{EEC52897-73DB-4F3B-9403-F15653D735D6}"/>
+    <hyperlink ref="A9" r:id="rId4" xr:uid="{96131781-1525-418D-85AB-FB1F70170CED}"/>
+    <hyperlink ref="A2" r:id="rId5" xr:uid="{CE4AEB79-F9AE-4730-BBED-8C26BF5D373C}"/>
+    <hyperlink ref="A13" r:id="rId6" xr:uid="{68E912E9-931C-4769-8998-8823509BE697}"/>
+    <hyperlink ref="A3" r:id="rId7" xr:uid="{42E071B9-30D8-4750-B517-BB6DCB7412DE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
changes for collection page suite
</commit_message>
<xml_diff>
--- a/src/main/resources/AllCollectionPages.xlsx
+++ b/src/main/resources/AllCollectionPages.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vijeta\git\TJ_Automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D47F69B-B8AA-48C7-B973-A8C18FCD3F65}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7834F67-AECB-4F68-925F-B4E45A31BB0F}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
   <si>
     <t>https://tommyjohn.com/collections/mens-new-arrivals-1</t>
   </si>
@@ -246,27 +246,6 @@
     <t>https://tommyjohn.com/collections/womens-lounge-sleep-packs</t>
   </si>
   <si>
-    <t>https://tommyjohn.com/collections/womens-sale-underwear</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/womens-sale-lounge-sleep</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/womens-sale-tops-tees</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/womens-sale-joggers</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/womens-sale-sweaters-jackets</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/womens-sale-camisoles</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/womens-sale-clothing</t>
-  </si>
-  <si>
     <t>https://tommyjohn.com/collections/womens-tops-tees</t>
   </si>
   <si>
@@ -277,9 +256,6 @@
   </si>
   <si>
     <t>https://tommyjohn.com/collections/womens-all-socks</t>
-  </si>
-  <si>
-    <t>https://tommyjohn.com/collections/mens-sale-pants-joggers</t>
   </si>
   <si>
     <t>https://tommyjohn.com/collections/womens-sale</t>
@@ -687,7 +663,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A98"/>
+  <dimension ref="A1:A90"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="98.54296875" bestFit="1" customWidth="1"/>
@@ -695,12 +671,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
@@ -710,7 +686,7 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
@@ -1035,152 +1011,112 @@
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>72</v>
+        <v>16</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>74</v>
+        <v>17</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>76</v>
+        <v>18</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>79</v>
+        <v>19</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>80</v>
+        <v>21</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>18</v>
+        <v>76</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>25</v>
+        <v>81</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>19</v>
+        <v>82</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>20</v>
+        <v>83</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>21</v>
+        <v>84</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>88</v>
-      </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A91" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A92" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A93" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A94" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A95" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A96" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A97" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A98" t="s">
-        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>